<commit_message>
Actualización cuadros / dibujo / acero
</commit_message>
<xml_diff>
--- a/ref/Placa Base/PB_VERIFICACIONES.xlsx
+++ b/ref/Placa Base/PB_VERIFICACIONES.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\10.10.0.30\Civil\03 - STD TEKLA\ref\Placa Base\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\03 - STD TEKLA\ref\Placa Base\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA3A5AC3-AAA1-485D-8898-FBBFB263229A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{993156C8-4DE6-49B3-B932-1C1CBC62283E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PB" sheetId="1" r:id="rId1"/>
@@ -295,7 +295,6 @@
         <name val="Arial"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="0" formatCode="General"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
@@ -362,30 +361,6 @@
     </dxf>
     <dxf>
       <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FF1F4E78"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
         <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
@@ -407,6 +382,22 @@
         </patternFill>
       </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFBFBFBF"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -424,6 +415,7 @@
         <name val="Arial"/>
         <scheme val="none"/>
       </font>
+      <numFmt numFmtId="0" formatCode="General"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
@@ -871,22 +863,30 @@
         </patternFill>
       </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FFBFBFBF"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFBFBFBF"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFBFBFBF"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFBFBFBF"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF1F4E78"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -902,27 +902,27 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E8367052-7810-4CA1-9C70-F48FA2998CC0}" name="Table1" displayName="Table1" ref="A1:O30" totalsRowShown="0" headerRowDxfId="2" dataDxfId="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E8367052-7810-4CA1-9C70-F48FA2998CC0}" name="Table1" displayName="Table1" ref="A1:O30" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
   <autoFilter ref="A1:O30" xr:uid="{E8367052-7810-4CA1-9C70-F48FA2998CC0}"/>
   <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{F50DDB28-7D44-48CC-B5E4-97688A435C4B}" name="Perfil" dataDxfId="15"/>
-    <tableColumn id="2" xr3:uid="{35C5EE2C-AEE7-4B69-9BF3-B2D0A827EA20}" name="Variante" dataDxfId="14"/>
-    <tableColumn id="3" xr3:uid="{9D59C8AF-EDEB-44CE-AC7B-393F6F67F352}" name="Etapa" dataDxfId="13"/>
-    <tableColumn id="4" xr3:uid="{2AB36A82-CB12-40DD-81A0-039A48826490}" name="Placa (mm)" dataDxfId="12"/>
-    <tableColumn id="5" xr3:uid="{A2C839AD-2B0A-402A-9B8E-08E4937E9FE4}" name="D anclaje" dataDxfId="11"/>
-    <tableColumn id="6" xr3:uid="{8C66F9C1-C32D-4CDD-867B-D238E01DFC92}" name="t placa (mm)" dataDxfId="10"/>
-    <tableColumn id="7" xr3:uid="{B41F9EB9-8820-4BF0-80A3-5CAF811BEE17}" name="h_ef (mm)" dataDxfId="9"/>
-    <tableColumn id="8" xr3:uid="{BFA1CBF2-CDCF-47DB-A0F5-B1641E80C69E}" name="Proy. sobre placa (mm)" dataDxfId="8"/>
-    <tableColumn id="9" xr3:uid="{55D39B72-64CD-4D9A-BBE5-EC0082C4FBE7}" name="s1 (mm) // d" dataDxfId="7"/>
-    <tableColumn id="10" xr3:uid="{231757F5-DDD4-45FE-8BA5-8AA9517A80A4}" name="s2 (mm) // bf" dataDxfId="6"/>
-    <tableColumn id="16" xr3:uid="{77E3C361-ACB2-41B6-9E69-00B7E3E82790}" name="s1 (mm) // redondeado" dataDxfId="0">
+    <tableColumn id="1" xr3:uid="{F50DDB28-7D44-48CC-B5E4-97688A435C4B}" name="Perfil" dataDxfId="13"/>
+    <tableColumn id="2" xr3:uid="{35C5EE2C-AEE7-4B69-9BF3-B2D0A827EA20}" name="Variante" dataDxfId="12"/>
+    <tableColumn id="3" xr3:uid="{9D59C8AF-EDEB-44CE-AC7B-393F6F67F352}" name="Etapa" dataDxfId="11"/>
+    <tableColumn id="4" xr3:uid="{2AB36A82-CB12-40DD-81A0-039A48826490}" name="Placa (mm)" dataDxfId="10"/>
+    <tableColumn id="5" xr3:uid="{A2C839AD-2B0A-402A-9B8E-08E4937E9FE4}" name="D anclaje" dataDxfId="9"/>
+    <tableColumn id="6" xr3:uid="{8C66F9C1-C32D-4CDD-867B-D238E01DFC92}" name="t placa (mm)" dataDxfId="8"/>
+    <tableColumn id="7" xr3:uid="{B41F9EB9-8820-4BF0-80A3-5CAF811BEE17}" name="h_ef (mm)" dataDxfId="7"/>
+    <tableColumn id="8" xr3:uid="{BFA1CBF2-CDCF-47DB-A0F5-B1641E80C69E}" name="Proy. sobre placa (mm)" dataDxfId="6"/>
+    <tableColumn id="9" xr3:uid="{55D39B72-64CD-4D9A-BBE5-EC0082C4FBE7}" name="s1 (mm) // d" dataDxfId="5"/>
+    <tableColumn id="10" xr3:uid="{231757F5-DDD4-45FE-8BA5-8AA9517A80A4}" name="s2 (mm) // bf" dataDxfId="4"/>
+    <tableColumn id="16" xr3:uid="{77E3C361-ACB2-41B6-9E69-00B7E3E82790}" name="s1 (mm) // redondeado" dataDxfId="3">
       <calculatedColumnFormula>+ROUNDUP(Table1[[#This Row],[s1 (mm) // d]],-1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="17" xr3:uid="{429B5AC0-DB41-4621-9EA4-3DA68D8031EB}" name="s2 (mm) // redondeado" dataDxfId="1">
+    <tableColumn id="17" xr3:uid="{429B5AC0-DB41-4621-9EA4-3DA68D8031EB}" name="s2 (mm) // redondeado" dataDxfId="2">
       <calculatedColumnFormula>+ROUNDUP(Table1[[#This Row],[s2 (mm) // bf]],-1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{9F453753-33C9-42EB-840E-543FF93A5659}" name="Rigidizadores" dataDxfId="5"/>
-    <tableColumn id="13" xr3:uid="{9A662CA9-9573-4ACA-B72C-F671E53AB467}" name="Arand. 2° (mm)" dataDxfId="4"/>
+    <tableColumn id="12" xr3:uid="{9F453753-33C9-42EB-840E-543FF93A5659}" name="Rigidizadores" dataDxfId="1"/>
+    <tableColumn id="13" xr3:uid="{9A662CA9-9573-4ACA-B72C-F671E53AB467}" name="Arand. 2° (mm)" dataDxfId="0"/>
     <tableColumn id="15" xr3:uid="{39D81073-7FBD-4316-A1E0-D3CD09A671CC}" name="Preset">
       <calculatedColumnFormula>+_xlfn.CONCAT(A2,"-",IF(B2="ARTICULADA","ART","EMP"),"-",C2)</calculatedColumnFormula>
     </tableColumn>
@@ -1217,24 +1217,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:O30"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.7109375" customWidth="1"/>
+    <col min="1" max="1" width="11.6640625" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="8.28515625" customWidth="1"/>
-    <col min="4" max="4" width="13.5703125" customWidth="1"/>
-    <col min="5" max="5" width="11.5703125" customWidth="1"/>
-    <col min="6" max="6" width="14.7109375" customWidth="1"/>
-    <col min="7" max="7" width="12.42578125" customWidth="1"/>
-    <col min="8" max="8" width="25.42578125" customWidth="1"/>
-    <col min="9" max="9" width="14.28515625" customWidth="1"/>
-    <col min="10" max="12" width="14.85546875" customWidth="1"/>
-    <col min="13" max="13" width="18.7109375" customWidth="1"/>
-    <col min="14" max="14" width="17.42578125" customWidth="1"/>
-    <col min="15" max="15" width="14.5703125" customWidth="1"/>
+    <col min="3" max="3" width="8.33203125" customWidth="1"/>
+    <col min="4" max="4" width="13.5546875" customWidth="1"/>
+    <col min="5" max="5" width="11.5546875" customWidth="1"/>
+    <col min="6" max="6" width="14.6640625" customWidth="1"/>
+    <col min="7" max="7" width="12.44140625" customWidth="1"/>
+    <col min="8" max="8" width="25.44140625" customWidth="1"/>
+    <col min="9" max="9" width="14.33203125" customWidth="1"/>
+    <col min="10" max="12" width="14.88671875" customWidth="1"/>
+    <col min="13" max="13" width="18.6640625" customWidth="1"/>
+    <col min="14" max="14" width="17.44140625" customWidth="1"/>
+    <col min="15" max="15" width="14.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" ht="32.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1281,7 +1281,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>12</v>
       </c>
@@ -1301,11 +1301,11 @@
         <v>19.100000000000001</v>
       </c>
       <c r="G2" s="2">
-        <f>+ROUNDUP(3/4*25.4*IF(B2="Articulada",12,18),-1)</f>
+        <f t="shared" ref="G2:G11" si="0">+ROUNDUP(3/4*25.4*IF(B2="Articulada",12,18),-1)</f>
         <v>230</v>
       </c>
       <c r="H2" s="2">
-        <v>86</v>
+        <v>60</v>
       </c>
       <c r="I2" s="2">
         <v>100</v>
@@ -1328,11 +1328,11 @@
         <v>18</v>
       </c>
       <c r="O2" t="str">
-        <f>+_xlfn.CONCAT(A2,"-",IF(B2="ARTICULADA","ART","EMP"),"-",C2)</f>
+        <f t="shared" ref="O2:O30" si="1">+_xlfn.CONCAT(A2,"-",IF(B2="ARTICULADA","ART","EMP"),"-",C2)</f>
         <v>W6x15-ART-1°</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -1352,11 +1352,11 @@
         <v>19.100000000000001</v>
       </c>
       <c r="G3" s="2">
-        <f>+ROUNDUP(3/4*25.4*IF(B3="Articulada",12,18),-1)</f>
+        <f t="shared" si="0"/>
         <v>350</v>
       </c>
       <c r="H3" s="2">
-        <v>86</v>
+        <v>60</v>
       </c>
       <c r="I3" s="2">
         <v>243</v>
@@ -1379,11 +1379,11 @@
         <v>18</v>
       </c>
       <c r="O3" t="str">
-        <f>+_xlfn.CONCAT(A3,"-",IF(B3="ARTICULADA","ART","EMP"),"-",C3)</f>
+        <f t="shared" si="1"/>
         <v>W6x15-EMP-1°</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>12</v>
       </c>
@@ -1403,11 +1403,11 @@
         <v>19.100000000000001</v>
       </c>
       <c r="G4" s="2">
-        <f>+ROUNDUP(3/4*25.4*IF(B4="Articulada",12,18),-1)</f>
+        <f t="shared" si="0"/>
         <v>350</v>
       </c>
       <c r="H4" s="2">
-        <v>86</v>
+        <v>60</v>
       </c>
       <c r="I4" s="2">
         <v>293</v>
@@ -1430,11 +1430,11 @@
         <v>20</v>
       </c>
       <c r="O4" t="str">
-        <f>+_xlfn.CONCAT(A4,"-",IF(B4="ARTICULADA","ART","EMP"),"-",C4)</f>
+        <f t="shared" si="1"/>
         <v>W6x15-EMP-2°</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>25</v>
       </c>
@@ -1454,11 +1454,11 @@
         <v>19.100000000000001</v>
       </c>
       <c r="G5" s="2">
-        <f>+ROUNDUP(3/4*25.4*IF(B5="Articulada",12,18),-1)</f>
+        <f t="shared" si="0"/>
         <v>230</v>
       </c>
-      <c r="H5" s="3">
-        <v>86</v>
+      <c r="H5" s="2">
+        <v>60</v>
       </c>
       <c r="I5" s="3">
         <v>150</v>
@@ -1481,11 +1481,11 @@
         <v>18</v>
       </c>
       <c r="O5" t="str">
-        <f>+_xlfn.CONCAT(A5,"-",IF(B5="ARTICULADA","ART","EMP"),"-",C5)</f>
+        <f t="shared" si="1"/>
         <v>W8x18-ART-1°</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>25</v>
       </c>
@@ -1505,11 +1505,11 @@
         <v>19.100000000000001</v>
       </c>
       <c r="G6" s="2">
-        <f>+ROUNDUP(3/4*25.4*IF(B6="Articulada",12,18),-1)</f>
+        <f t="shared" si="0"/>
         <v>350</v>
       </c>
-      <c r="H6" s="3">
-        <v>86</v>
+      <c r="H6" s="2">
+        <v>60</v>
       </c>
       <c r="I6" s="3">
         <v>293</v>
@@ -1532,11 +1532,11 @@
         <v>18</v>
       </c>
       <c r="O6" t="str">
-        <f>+_xlfn.CONCAT(A6,"-",IF(B6="ARTICULADA","ART","EMP"),"-",C6)</f>
+        <f t="shared" si="1"/>
         <v>W8x18-EMP-1°</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>25</v>
       </c>
@@ -1556,11 +1556,11 @@
         <v>19.100000000000001</v>
       </c>
       <c r="G7" s="2">
-        <f>+ROUNDUP(3/4*25.4*IF(B7="Articulada",12,18),-1)</f>
+        <f t="shared" si="0"/>
         <v>350</v>
       </c>
-      <c r="H7" s="3">
-        <v>86</v>
+      <c r="H7" s="2">
+        <v>60</v>
       </c>
       <c r="I7" s="3">
         <v>343</v>
@@ -1583,11 +1583,11 @@
         <v>20</v>
       </c>
       <c r="O7" t="str">
-        <f>+_xlfn.CONCAT(A7,"-",IF(B7="ARTICULADA","ART","EMP"),"-",C7)</f>
+        <f t="shared" si="1"/>
         <v>W8x18-EMP-2°</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>28</v>
       </c>
@@ -1607,11 +1607,11 @@
         <v>19.100000000000001</v>
       </c>
       <c r="G8" s="2">
-        <f>+ROUNDUP(3/4*25.4*IF(B8="Articulada",12,18),-1)</f>
+        <f t="shared" si="0"/>
         <v>230</v>
       </c>
       <c r="H8" s="2">
-        <v>86</v>
+        <v>60</v>
       </c>
       <c r="I8" s="2">
         <v>150</v>
@@ -1634,11 +1634,11 @@
         <v>18</v>
       </c>
       <c r="O8" t="str">
-        <f>+_xlfn.CONCAT(A8,"-",IF(B8="ARTICULADA","ART","EMP"),"-",C8)</f>
+        <f t="shared" si="1"/>
         <v>W8x31-ART-1°</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>28</v>
       </c>
@@ -1658,11 +1658,11 @@
         <v>19.100000000000001</v>
       </c>
       <c r="G9" s="2">
-        <f>+ROUNDUP(3/4*25.4*IF(B9="Articulada",12,18),-1)</f>
+        <f t="shared" si="0"/>
         <v>230</v>
       </c>
       <c r="H9" s="2">
-        <v>86</v>
+        <v>60</v>
       </c>
       <c r="I9" s="2">
         <v>150</v>
@@ -1685,11 +1685,11 @@
         <v>20</v>
       </c>
       <c r="O9" t="str">
-        <f>+_xlfn.CONCAT(A9,"-",IF(B9="ARTICULADA","ART","EMP"),"-",C9)</f>
+        <f t="shared" si="1"/>
         <v>W8x31-ART-2°</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>28</v>
       </c>
@@ -1709,11 +1709,11 @@
         <v>19.100000000000001</v>
       </c>
       <c r="G10" s="2">
-        <f>+ROUNDUP(3/4*25.4*IF(B10="Articulada",12,18),-1)</f>
+        <f t="shared" si="0"/>
         <v>350</v>
       </c>
       <c r="H10" s="2">
-        <v>86</v>
+        <v>60</v>
       </c>
       <c r="I10" s="2">
         <v>293</v>
@@ -1736,11 +1736,11 @@
         <v>18</v>
       </c>
       <c r="O10" t="str">
-        <f>+_xlfn.CONCAT(A10,"-",IF(B10="ARTICULADA","ART","EMP"),"-",C10)</f>
+        <f t="shared" si="1"/>
         <v>W8x31-EMP-1°</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>28</v>
       </c>
@@ -1760,11 +1760,11 @@
         <v>19.100000000000001</v>
       </c>
       <c r="G11" s="2">
-        <f>+ROUNDUP(3/4*25.4*IF(B11="Articulada",12,18),-1)</f>
+        <f t="shared" si="0"/>
         <v>350</v>
       </c>
       <c r="H11" s="2">
-        <v>86</v>
+        <v>60</v>
       </c>
       <c r="I11" s="2">
         <v>343</v>
@@ -1787,11 +1787,11 @@
         <v>20</v>
       </c>
       <c r="O11" t="str">
-        <f>+_xlfn.CONCAT(A11,"-",IF(B11="ARTICULADA","ART","EMP"),"-",C11)</f>
+        <f t="shared" si="1"/>
         <v>W8x31-EMP-2°</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>29</v>
       </c>
@@ -1811,7 +1811,7 @@
         <v>25.4</v>
       </c>
       <c r="G12" s="2">
-        <f>+ROUNDUP(25.4*IF(B12="Articulada",12,18),-1)</f>
+        <f t="shared" ref="G12:G18" si="2">+ROUNDUP(25.4*IF(B12="Articulada",12,18),-1)</f>
         <v>310</v>
       </c>
       <c r="H12" s="3">
@@ -1838,11 +1838,11 @@
         <v>18</v>
       </c>
       <c r="O12" t="str">
-        <f>+_xlfn.CONCAT(A12,"-",IF(B12="ARTICULADA","ART","EMP"),"-",C12)</f>
+        <f t="shared" si="1"/>
         <v>W10x45-ART-1°</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>29</v>
       </c>
@@ -1862,7 +1862,7 @@
         <v>25.4</v>
       </c>
       <c r="G13" s="2">
-        <f>+ROUNDUP(25.4*IF(B13="Articulada",12,18),-1)</f>
+        <f t="shared" si="2"/>
         <v>460</v>
       </c>
       <c r="H13" s="3">
@@ -1889,11 +1889,11 @@
         <v>18</v>
       </c>
       <c r="O13" t="str">
-        <f>+_xlfn.CONCAT(A13,"-",IF(B13="ARTICULADA","ART","EMP"),"-",C13)</f>
+        <f t="shared" si="1"/>
         <v>W10x45-EMP-1°</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
         <v>29</v>
       </c>
@@ -1913,7 +1913,7 @@
         <v>25.4</v>
       </c>
       <c r="G14" s="2">
-        <f>+ROUNDUP(25.4*IF(B14="Articulada",12,18),-1)</f>
+        <f t="shared" si="2"/>
         <v>460</v>
       </c>
       <c r="H14" s="3">
@@ -1940,11 +1940,11 @@
         <v>31</v>
       </c>
       <c r="O14" t="str">
-        <f>+_xlfn.CONCAT(A14,"-",IF(B14="ARTICULADA","ART","EMP"),"-",C14)</f>
+        <f t="shared" si="1"/>
         <v>W10x45-EMP-2°</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>33</v>
       </c>
@@ -1964,7 +1964,7 @@
         <v>25.4</v>
       </c>
       <c r="G15" s="2">
-        <f>+ROUNDUP(25.4*IF(B15="Articulada",12,18),-1)</f>
+        <f t="shared" si="2"/>
         <v>310</v>
       </c>
       <c r="H15" s="2">
@@ -1991,11 +1991,11 @@
         <v>18</v>
       </c>
       <c r="O15" t="str">
-        <f>+_xlfn.CONCAT(A15,"-",IF(B15="ARTICULADA","ART","EMP"),"-",C15)</f>
+        <f t="shared" si="1"/>
         <v>W12x50-ART-1°</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>33</v>
       </c>
@@ -2015,7 +2015,7 @@
         <v>25.4</v>
       </c>
       <c r="G16" s="2">
-        <f>+ROUNDUP(25.4*IF(B16="Articulada",12,18),-1)</f>
+        <f t="shared" si="2"/>
         <v>460</v>
       </c>
       <c r="H16" s="2">
@@ -2042,11 +2042,11 @@
         <v>18</v>
       </c>
       <c r="O16" t="str">
-        <f>+_xlfn.CONCAT(A16,"-",IF(B16="ARTICULADA","ART","EMP"),"-",C16)</f>
+        <f t="shared" si="1"/>
         <v>W12x50-EMP-1°</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
         <v>34</v>
       </c>
@@ -2066,7 +2066,7 @@
         <v>25.4</v>
       </c>
       <c r="G17" s="2">
-        <f>+ROUNDUP(25.4*IF(B17="Articulada",12,18),-1)</f>
+        <f t="shared" si="2"/>
         <v>310</v>
       </c>
       <c r="H17" s="3">
@@ -2093,11 +2093,11 @@
         <v>18</v>
       </c>
       <c r="O17" t="str">
-        <f>+_xlfn.CONCAT(A17,"-",IF(B17="ARTICULADA","ART","EMP"),"-",C17)</f>
+        <f t="shared" si="1"/>
         <v>W14x74-ART-1°</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
         <v>34</v>
       </c>
@@ -2117,7 +2117,7 @@
         <v>25.4</v>
       </c>
       <c r="G18" s="2">
-        <f>+ROUNDUP(25.4*IF(B18="Articulada",12,18),-1)</f>
+        <f t="shared" si="2"/>
         <v>460</v>
       </c>
       <c r="H18" s="3">
@@ -2144,11 +2144,11 @@
         <v>18</v>
       </c>
       <c r="O18" t="str">
-        <f>+_xlfn.CONCAT(A18,"-",IF(B18="ARTICULADA","ART","EMP"),"-",C18)</f>
+        <f t="shared" si="1"/>
         <v>W14x74-EMP-1°</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>35</v>
       </c>
@@ -2195,11 +2195,11 @@
         <v>18</v>
       </c>
       <c r="O19" t="str">
-        <f>+_xlfn.CONCAT(A19,"-",IF(B19="ARTICULADA","ART","EMP"),"-",C19)</f>
+        <f t="shared" si="1"/>
         <v>HEB160-ART-1°</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>35</v>
       </c>
@@ -2246,11 +2246,11 @@
         <v>18</v>
       </c>
       <c r="O20" t="str">
-        <f>+_xlfn.CONCAT(A20,"-",IF(B20="ARTICULADA","ART","EMP"),"-",C20)</f>
+        <f t="shared" si="1"/>
         <v>HEB160-EMP-1°</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>35</v>
       </c>
@@ -2297,11 +2297,11 @@
         <v>20</v>
       </c>
       <c r="O21" t="str">
-        <f>+_xlfn.CONCAT(A21,"-",IF(B21="ARTICULADA","ART","EMP"),"-",C21)</f>
+        <f t="shared" si="1"/>
         <v>HEB160-EMP-2°</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
         <v>36</v>
       </c>
@@ -2348,11 +2348,11 @@
         <v>18</v>
       </c>
       <c r="O22" t="str">
-        <f>+_xlfn.CONCAT(A22,"-",IF(B22="ARTICULADA","ART","EMP"),"-",C22)</f>
+        <f t="shared" si="1"/>
         <v>HEB200-ART-1°</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
         <v>36</v>
       </c>
@@ -2399,11 +2399,11 @@
         <v>18</v>
       </c>
       <c r="O23" t="str">
-        <f>+_xlfn.CONCAT(A23,"-",IF(B23="ARTICULADA","ART","EMP"),"-",C23)</f>
+        <f t="shared" si="1"/>
         <v>HEB200-EMP-1°</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
         <v>36</v>
       </c>
@@ -2450,11 +2450,11 @@
         <v>31</v>
       </c>
       <c r="O24" t="str">
-        <f>+_xlfn.CONCAT(A24,"-",IF(B24="ARTICULADA","ART","EMP"),"-",C24)</f>
+        <f t="shared" si="1"/>
         <v>HEB200-EMP-2°</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>45</v>
       </c>
@@ -2501,11 +2501,11 @@
         <v>18</v>
       </c>
       <c r="O25" t="str">
-        <f>+_xlfn.CONCAT(A25,"-",IF(B25="ARTICULADA","ART","EMP"),"-",C25)</f>
+        <f t="shared" si="1"/>
         <v>UPN140C-EMP-1°</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>45</v>
       </c>
@@ -2552,11 +2552,11 @@
         <v>20</v>
       </c>
       <c r="O26" t="str">
-        <f>+_xlfn.CONCAT(A26,"-",IF(B26="ARTICULADA","ART","EMP"),"-",C26)</f>
+        <f t="shared" si="1"/>
         <v>UPN140C-EMP-2°</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
         <v>46</v>
       </c>
@@ -2603,11 +2603,11 @@
         <v>18</v>
       </c>
       <c r="O27" t="str">
-        <f>+_xlfn.CONCAT(A27,"-",IF(B27="ARTICULADA","ART","EMP"),"-",C27)</f>
+        <f t="shared" si="1"/>
         <v>UPN180C-EMP-1°</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A28" s="3" t="s">
         <v>46</v>
       </c>
@@ -2654,11 +2654,11 @@
         <v>20</v>
       </c>
       <c r="O28" t="str">
-        <f>+_xlfn.CONCAT(A28,"-",IF(B28="ARTICULADA","ART","EMP"),"-",C28)</f>
+        <f t="shared" si="1"/>
         <v>UPN180C-EMP-2°</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>47</v>
       </c>
@@ -2705,11 +2705,11 @@
         <v>18</v>
       </c>
       <c r="O29" t="str">
-        <f>+_xlfn.CONCAT(A29,"-",IF(B29="ARTICULADA","ART","EMP"),"-",C29)</f>
+        <f t="shared" si="1"/>
         <v>UPN220C-EMP-1°</v>
       </c>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>47</v>
       </c>
@@ -2756,7 +2756,7 @@
         <v>31</v>
       </c>
       <c r="O30" t="str">
-        <f>+_xlfn.CONCAT(A30,"-",IF(B30="ARTICULADA","ART","EMP"),"-",C30)</f>
+        <f t="shared" si="1"/>
         <v>UPN220C-EMP-2°</v>
       </c>
     </row>

</xml_diff>